<commit_message>
Catalogue: regenerate go-live seed from updated Title Master (251 titles)
</commit_message>
<xml_diff>
--- a/backend/title_master_go_live.xlsx
+++ b/backend/title_master_go_live.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e94e64837a8caf2a/Desktop/Renu Mar 26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{08F30001-AB10-4607-85E9-90C343CEEFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54AF753C-FF8C-4EE7-9544-12793003EB1C}"/>
+  <xr:revisionPtr revIDLastSave="147" documentId="13_ncr:1_{08F30001-AB10-4607-85E9-90C343CEEFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06D36A9D-D550-4759-916B-35B2C9ADBB0D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5E621DD9-F29B-40CE-88A2-F27056FA0A8E}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AF$248</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AF$252</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2328" uniqueCount="953">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2364" uniqueCount="966">
   <si>
     <t>Subject</t>
   </si>
@@ -4233,12 +4233,51 @@
     <t>Shishir Priyadarshi is the President of Chintan Research Foundation. He is a former WTO Director with around twenty-five years of experience in international trade, economic policy, and developmental issues. As a former IAS officer, he served in senior positions in India, both at the federal and subfederal levels, including in the office of the Cabinet Secretary. He has published extensively, held academic affiliations worldwide, and remains committed to sustainable and inclusive development. He has also written several articles &amp; opinion pieces on public policy issues, this edited book being an example of that.
 Dr Cchavi Vasisht is an Associate Fellow at the Centre for Geopolitics and Strategic Studies. She has been awarded her PhD thesis titled “Women Entrepreneurs in Nepal” from the Centre for South Asian Studies, School of International Studies, Jawaharlal Nehru University. She has been awarded the UGC NET Senior Research Fellowship to pursue her research work. She has a keen interest in the geopolitics of South Asia, Southeast Asia, particularly Myanmar, and Gender related issues. She has also co-edited books, titled “Revisiting Myanmar” along with Brig Vinod Anand and “Perspectives from and Within India and its Neighbourhood” with Shishir Priyadarshi.</t>
   </si>
+  <si>
+    <t>Legal Aptitude &amp; Reasoning LA/LR  2/e (2026-27)</t>
+  </si>
+  <si>
+    <t>Climate Justice</t>
+  </si>
+  <si>
+    <t>Sudhir Mishra</t>
+  </si>
+  <si>
+    <t>Corporate Law Referencer 12/e</t>
+  </si>
+  <si>
+    <t>In-House Matters</t>
+  </si>
+  <si>
+    <t>Pramod Rao</t>
+  </si>
+  <si>
+    <t>Legal Aptitude &amp; Reasoning (LA/LR) for CLAT, AILET, SLAT and Other Law Entrance Tests is a comprehensive book on legal reasoning designed for law entrance exam preparation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishrut Jain is a graduate of the West Bengal National University of Juridical Sciences (NUJS), Kolkata. </t>
+  </si>
+  <si>
+    <t>The in-house counsel, once a go-between, now sits at the table where decisions are made: advising boards, shaping strategy, steering companies through complexity and change.</t>
+  </si>
+  <si>
+    <t>Pramod Rao is a former Executive Director at the Securities and Exchange Board of India (SEBI), and former Board Member of IFSCA, NFRA, and IICA.</t>
+  </si>
+  <si>
+    <t>eMinds Legal is a boutique Corporate Law Firm based in Gurgaon, India, specializing in Corporate Secretarial, Corporate Legal, Compliance, Accounting &amp; Payroll.</t>
+  </si>
+  <si>
+    <t>Climate Justice: 75 Years of Supreme Court —75 Judgments that Built Climate Jurisprudence in India is more than a legal compendium; it is a journey through seventy-five carefully selected judgments that reveal the evolution of India’s environmental consciousness.</t>
+  </si>
+  <si>
+    <t>Mr. Sudhir Mishra is a leading disputes and climate change lawyer and a Door Tenant at No.5 Barristers’ Chambers, UK.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4378,6 +4417,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -4405,7 +4452,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -4441,11 +4488,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -4558,15 +4618,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
@@ -4597,6 +4648,51 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="17" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4612,10 +4708,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4915,12 +5007,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAB18B99-872A-4F67-B7AF-943353254B42}">
-  <dimension ref="A1:AF249"/>
+  <dimension ref="A1:AF255"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.140625" style="1" customWidth="1"/>
     <col min="2" max="3" width="12.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" style="3" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="19.42578125" style="1" customWidth="1"/>
     <col min="7" max="7" width="33.5703125" style="1" customWidth="1"/>
@@ -4932,7 +5024,7 @@
     <col min="13" max="13" width="20.85546875" style="1" customWidth="1"/>
     <col min="14" max="14" width="20.7109375" style="1" customWidth="1"/>
     <col min="15" max="15" width="10.7109375" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15" style="50" customWidth="1"/>
+    <col min="16" max="16" width="15" style="47" customWidth="1"/>
     <col min="17" max="17" width="11.85546875" style="1" customWidth="1"/>
     <col min="18" max="18" width="11.42578125" style="1" customWidth="1"/>
     <col min="19" max="19" width="11.7109375" style="1" customWidth="1"/>
@@ -4986,7 +5078,7 @@
       <c r="O1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="46" t="s">
+      <c r="P1" s="43" t="s">
         <v>10</v>
       </c>
       <c r="Q1" s="2" t="s">
@@ -5059,7 +5151,7 @@
         <f>38+261</f>
         <v>299</v>
       </c>
-      <c r="P2" s="47">
+      <c r="P2" s="44">
         <v>295</v>
       </c>
       <c r="Q2" s="6">
@@ -5122,7 +5214,7 @@
         <f>214+24</f>
         <v>238</v>
       </c>
-      <c r="P3" s="47">
+      <c r="P3" s="44">
         <v>650</v>
       </c>
       <c r="Q3" s="6">
@@ -5185,7 +5277,7 @@
         <f>34+288</f>
         <v>322</v>
       </c>
-      <c r="P4" s="47">
+      <c r="P4" s="44">
         <v>695</v>
       </c>
       <c r="Q4" s="6">
@@ -5248,7 +5340,7 @@
         <f>247+12</f>
         <v>259</v>
       </c>
-      <c r="P5" s="47">
+      <c r="P5" s="44">
         <v>275</v>
       </c>
       <c r="Q5" s="31">
@@ -5311,7 +5403,7 @@
         <f>302+32</f>
         <v>334</v>
       </c>
-      <c r="P6" s="47">
+      <c r="P6" s="44">
         <v>1195</v>
       </c>
       <c r="Q6" s="6">
@@ -5374,7 +5466,7 @@
         <f>536+34+162</f>
         <v>732</v>
       </c>
-      <c r="P7" s="47">
+      <c r="P7" s="44">
         <v>1250</v>
       </c>
       <c r="Q7" s="6">
@@ -5437,7 +5529,7 @@
         <f>230+16</f>
         <v>246</v>
       </c>
-      <c r="P8" s="47">
+      <c r="P8" s="44">
         <v>275</v>
       </c>
       <c r="Q8" s="6">
@@ -5500,7 +5592,7 @@
         <f>303+19</f>
         <v>322</v>
       </c>
-      <c r="P9" s="47">
+      <c r="P9" s="44">
         <v>350</v>
       </c>
       <c r="Q9" s="6">
@@ -5563,7 +5655,7 @@
         <f>508+26</f>
         <v>534</v>
       </c>
-      <c r="P10" s="47">
+      <c r="P10" s="44">
         <v>695</v>
       </c>
       <c r="Q10" s="6">
@@ -5626,7 +5718,7 @@
         <f>366+30</f>
         <v>396</v>
       </c>
-      <c r="P11" s="47">
+      <c r="P11" s="44">
         <v>895</v>
       </c>
       <c r="Q11" s="6">
@@ -5689,7 +5781,7 @@
         <f>108+28</f>
         <v>136</v>
       </c>
-      <c r="P12" s="47">
+      <c r="P12" s="44">
         <v>350</v>
       </c>
       <c r="Q12" s="6">
@@ -5752,7 +5844,7 @@
         <f>452+12</f>
         <v>464</v>
       </c>
-      <c r="P13" s="47">
+      <c r="P13" s="44">
         <v>575</v>
       </c>
       <c r="Q13" s="6">
@@ -5815,7 +5907,7 @@
         <f>332+150</f>
         <v>482</v>
       </c>
-      <c r="P14" s="47">
+      <c r="P14" s="44">
         <v>995</v>
       </c>
       <c r="Q14" s="6">
@@ -5878,7 +5970,7 @@
         <f>270+16</f>
         <v>286</v>
       </c>
-      <c r="P15" s="47">
+      <c r="P15" s="44">
         <v>395</v>
       </c>
       <c r="Q15" s="6">
@@ -5941,7 +6033,7 @@
         <f>374+16</f>
         <v>390</v>
       </c>
-      <c r="P16" s="47">
+      <c r="P16" s="44">
         <v>295</v>
       </c>
       <c r="Q16" s="6">
@@ -6004,7 +6096,7 @@
         <f>254+18</f>
         <v>272</v>
       </c>
-      <c r="P17" s="47">
+      <c r="P17" s="44">
         <v>450</v>
       </c>
       <c r="Q17" s="6">
@@ -6067,7 +6159,7 @@
         <f>294+14</f>
         <v>308</v>
       </c>
-      <c r="P18" s="47">
+      <c r="P18" s="44">
         <v>295</v>
       </c>
       <c r="Q18" s="6">
@@ -6130,7 +6222,7 @@
         <f>324+12</f>
         <v>336</v>
       </c>
-      <c r="P19" s="47">
+      <c r="P19" s="44">
         <v>295</v>
       </c>
       <c r="Q19" s="6">
@@ -6192,7 +6284,7 @@
       <c r="O20" s="4">
         <v>464</v>
       </c>
-      <c r="P20" s="47">
+      <c r="P20" s="44">
         <v>695</v>
       </c>
       <c r="Q20" s="6">
@@ -6255,7 +6347,7 @@
         <f>260+34</f>
         <v>294</v>
       </c>
-      <c r="P21" s="47">
+      <c r="P21" s="44">
         <v>550</v>
       </c>
       <c r="Q21" s="6">
@@ -6318,7 +6410,7 @@
         <f>678+1038</f>
         <v>1716</v>
       </c>
-      <c r="P22" s="47">
+      <c r="P22" s="44">
         <v>2495</v>
       </c>
       <c r="Q22" s="6">
@@ -6381,7 +6473,7 @@
         <f>354+14</f>
         <v>368</v>
       </c>
-      <c r="P23" s="47">
+      <c r="P23" s="44">
         <v>395</v>
       </c>
       <c r="Q23" s="6">
@@ -6444,7 +6536,7 @@
         <f>508+24</f>
         <v>532</v>
       </c>
-      <c r="P24" s="47">
+      <c r="P24" s="44">
         <v>1295</v>
       </c>
       <c r="Q24" s="6">
@@ -6507,7 +6599,7 @@
         <f>220+20</f>
         <v>240</v>
       </c>
-      <c r="P25" s="47">
+      <c r="P25" s="44">
         <v>295</v>
       </c>
       <c r="Q25" s="6">
@@ -6570,7 +6662,7 @@
         <f>198+20</f>
         <v>218</v>
       </c>
-      <c r="P26" s="47">
+      <c r="P26" s="44">
         <v>495</v>
       </c>
       <c r="Q26" s="6">
@@ -6633,7 +6725,7 @@
         <f>258+28</f>
         <v>286</v>
       </c>
-      <c r="P27" s="47">
+      <c r="P27" s="44">
         <v>895</v>
       </c>
       <c r="Q27" s="6">
@@ -6696,7 +6788,7 @@
         <f>432+24</f>
         <v>456</v>
       </c>
-      <c r="P28" s="47">
+      <c r="P28" s="44">
         <v>895</v>
       </c>
       <c r="Q28" s="6">
@@ -6759,7 +6851,7 @@
         <f>256+30</f>
         <v>286</v>
       </c>
-      <c r="P29" s="47">
+      <c r="P29" s="44">
         <v>795</v>
       </c>
       <c r="Q29" s="6">
@@ -6822,7 +6914,7 @@
         <f>312+26</f>
         <v>338</v>
       </c>
-      <c r="P30" s="47">
+      <c r="P30" s="44">
         <v>350</v>
       </c>
       <c r="Q30" s="6">
@@ -6884,7 +6976,7 @@
       <c r="O31" s="4">
         <v>252</v>
       </c>
-      <c r="P31" s="47">
+      <c r="P31" s="44">
         <v>295</v>
       </c>
       <c r="Q31" s="6">
@@ -6946,7 +7038,7 @@
       <c r="O32" s="4">
         <v>402</v>
       </c>
-      <c r="P32" s="47">
+      <c r="P32" s="44">
         <v>350</v>
       </c>
       <c r="Q32" s="6">
@@ -7008,7 +7100,7 @@
       <c r="O33" s="4">
         <v>292</v>
       </c>
-      <c r="P33" s="47">
+      <c r="P33" s="44">
         <v>295</v>
       </c>
       <c r="Q33" s="6">
@@ -7070,7 +7162,7 @@
       <c r="O34" s="4">
         <v>256</v>
       </c>
-      <c r="P34" s="47">
+      <c r="P34" s="44">
         <v>995</v>
       </c>
       <c r="Q34" s="6">
@@ -7132,7 +7224,7 @@
       <c r="O35" s="4">
         <v>304</v>
       </c>
-      <c r="P35" s="47">
+      <c r="P35" s="44">
         <v>295</v>
       </c>
       <c r="Q35" s="6">
@@ -7194,7 +7286,7 @@
       <c r="O36" s="4">
         <v>300</v>
       </c>
-      <c r="P36" s="47">
+      <c r="P36" s="44">
         <v>250</v>
       </c>
       <c r="Q36" s="6">
@@ -7256,7 +7348,7 @@
       <c r="O37" s="4">
         <v>354</v>
       </c>
-      <c r="P37" s="47">
+      <c r="P37" s="44">
         <v>950</v>
       </c>
       <c r="Q37" s="6">
@@ -7318,7 +7410,7 @@
       <c r="O38" s="4">
         <v>225</v>
       </c>
-      <c r="P38" s="47">
+      <c r="P38" s="44">
         <v>250</v>
       </c>
       <c r="Q38" s="6">
@@ -7380,7 +7472,7 @@
       <c r="O39" s="4">
         <v>298</v>
       </c>
-      <c r="P39" s="47">
+      <c r="P39" s="44">
         <v>295</v>
       </c>
       <c r="Q39" s="6">
@@ -7442,7 +7534,7 @@
       <c r="O40" s="4">
         <v>490</v>
       </c>
-      <c r="P40" s="47">
+      <c r="P40" s="44">
         <v>950</v>
       </c>
       <c r="Q40" s="6">
@@ -7504,7 +7596,7 @@
       <c r="O41" s="4">
         <v>320</v>
       </c>
-      <c r="P41" s="47">
+      <c r="P41" s="44">
         <v>295</v>
       </c>
       <c r="Q41" s="6">
@@ -7566,7 +7658,7 @@
       <c r="O42" s="4">
         <v>438</v>
       </c>
-      <c r="P42" s="47">
+      <c r="P42" s="44">
         <v>325</v>
       </c>
       <c r="Q42" s="6">
@@ -7628,7 +7720,7 @@
       <c r="O43" s="4">
         <v>872</v>
       </c>
-      <c r="P43" s="47">
+      <c r="P43" s="44">
         <v>1695</v>
       </c>
       <c r="Q43" s="6">
@@ -7690,7 +7782,7 @@
       <c r="O44" s="4">
         <v>484</v>
       </c>
-      <c r="P44" s="47">
+      <c r="P44" s="44">
         <v>450</v>
       </c>
       <c r="Q44" s="6">
@@ -7752,7 +7844,7 @@
       <c r="O45" s="4">
         <v>338</v>
       </c>
-      <c r="P45" s="47">
+      <c r="P45" s="44">
         <v>345</v>
       </c>
       <c r="Q45" s="6">
@@ -7814,7 +7906,7 @@
       <c r="O46" s="4">
         <v>380</v>
       </c>
-      <c r="P46" s="47">
+      <c r="P46" s="44">
         <v>795</v>
       </c>
       <c r="Q46" s="6">
@@ -7876,7 +7968,7 @@
       <c r="O47" s="4">
         <v>352</v>
       </c>
-      <c r="P47" s="47">
+      <c r="P47" s="44">
         <v>795</v>
       </c>
       <c r="Q47" s="6">
@@ -7938,7 +8030,7 @@
       <c r="O48" s="4">
         <v>590</v>
       </c>
-      <c r="P48" s="47">
+      <c r="P48" s="44">
         <v>595</v>
       </c>
       <c r="Q48" s="6">
@@ -8000,7 +8092,7 @@
       <c r="O49" s="4">
         <v>246</v>
       </c>
-      <c r="P49" s="47">
+      <c r="P49" s="44">
         <v>250</v>
       </c>
       <c r="Q49" s="6">
@@ -8062,7 +8154,7 @@
       <c r="O50" s="4">
         <v>236</v>
       </c>
-      <c r="P50" s="47">
+      <c r="P50" s="44">
         <v>495</v>
       </c>
       <c r="Q50" s="6">
@@ -8124,7 +8216,7 @@
       <c r="O51" s="4">
         <v>154</v>
       </c>
-      <c r="P51" s="47">
+      <c r="P51" s="44">
         <v>295</v>
       </c>
       <c r="Q51" s="6">
@@ -8186,7 +8278,7 @@
       <c r="O52" s="4">
         <v>516</v>
       </c>
-      <c r="P52" s="47">
+      <c r="P52" s="44">
         <v>995</v>
       </c>
       <c r="Q52" s="6">
@@ -8248,7 +8340,7 @@
       <c r="O53" s="4">
         <v>364</v>
       </c>
-      <c r="P53" s="47">
+      <c r="P53" s="44">
         <v>995</v>
       </c>
       <c r="Q53" s="6">
@@ -8310,7 +8402,7 @@
       <c r="O54" s="4">
         <v>892</v>
       </c>
-      <c r="P54" s="47">
+      <c r="P54" s="44">
         <v>1495</v>
       </c>
       <c r="Q54" s="6">
@@ -8372,7 +8464,7 @@
       <c r="O55" s="4">
         <v>460</v>
       </c>
-      <c r="P55" s="47">
+      <c r="P55" s="44">
         <v>375</v>
       </c>
       <c r="Q55" s="6">
@@ -8434,7 +8526,7 @@
       <c r="O56" s="4">
         <v>612</v>
       </c>
-      <c r="P56" s="47">
+      <c r="P56" s="44">
         <v>995</v>
       </c>
       <c r="Q56" s="6">
@@ -8496,7 +8588,7 @@
       <c r="O57" s="4">
         <v>346</v>
       </c>
-      <c r="P57" s="47">
+      <c r="P57" s="44">
         <v>1050</v>
       </c>
       <c r="Q57" s="6">
@@ -8558,7 +8650,7 @@
       <c r="O58" s="4">
         <v>816</v>
       </c>
-      <c r="P58" s="47">
+      <c r="P58" s="44">
         <v>795</v>
       </c>
       <c r="Q58" s="6">
@@ -8620,7 +8712,7 @@
       <c r="O59" s="4">
         <v>582</v>
       </c>
-      <c r="P59" s="47">
+      <c r="P59" s="44">
         <v>450</v>
       </c>
       <c r="Q59" s="6">
@@ -8682,7 +8774,7 @@
       <c r="O60" s="4">
         <v>244</v>
       </c>
-      <c r="P60" s="47">
+      <c r="P60" s="44">
         <v>295</v>
       </c>
       <c r="Q60" s="6">
@@ -8744,7 +8836,7 @@
       <c r="O61" s="4">
         <v>340</v>
       </c>
-      <c r="P61" s="47">
+      <c r="P61" s="44">
         <v>375</v>
       </c>
       <c r="Q61" s="6">
@@ -8806,7 +8898,7 @@
       <c r="O62" s="4">
         <v>395</v>
       </c>
-      <c r="P62" s="47">
+      <c r="P62" s="44">
         <v>395</v>
       </c>
       <c r="Q62" s="6">
@@ -8868,7 +8960,7 @@
       <c r="O63" s="4">
         <v>395</v>
       </c>
-      <c r="P63" s="47">
+      <c r="P63" s="44">
         <v>395</v>
       </c>
       <c r="Q63" s="6">
@@ -8930,7 +9022,7 @@
       <c r="O64" s="4">
         <v>395</v>
       </c>
-      <c r="P64" s="47">
+      <c r="P64" s="44">
         <v>395</v>
       </c>
       <c r="Q64" s="6">
@@ -8992,7 +9084,7 @@
       <c r="O65" s="4">
         <v>295</v>
       </c>
-      <c r="P65" s="47">
+      <c r="P65" s="44">
         <v>295</v>
       </c>
       <c r="Q65" s="6">
@@ -9054,7 +9146,7 @@
       <c r="O66" s="4">
         <v>360</v>
       </c>
-      <c r="P66" s="47">
+      <c r="P66" s="44">
         <v>795</v>
       </c>
       <c r="Q66" s="6">
@@ -9116,7 +9208,7 @@
       <c r="O67" s="4">
         <v>320</v>
       </c>
-      <c r="P67" s="47">
+      <c r="P67" s="44">
         <v>795</v>
       </c>
       <c r="Q67" s="6">
@@ -9178,7 +9270,7 @@
       <c r="O68" s="4">
         <v>272</v>
       </c>
-      <c r="P68" s="47">
+      <c r="P68" s="44">
         <v>795</v>
       </c>
       <c r="Q68" s="6">
@@ -9240,7 +9332,7 @@
       <c r="O69" s="4">
         <v>594</v>
       </c>
-      <c r="P69" s="47">
+      <c r="P69" s="44">
         <v>1595</v>
       </c>
       <c r="Q69" s="6">
@@ -9302,7 +9394,7 @@
       <c r="O70" s="4">
         <v>610</v>
       </c>
-      <c r="P70" s="47">
+      <c r="P70" s="44">
         <v>550</v>
       </c>
       <c r="Q70" s="6">
@@ -9364,7 +9456,7 @@
       <c r="O71" s="4">
         <v>278</v>
       </c>
-      <c r="P71" s="47">
+      <c r="P71" s="44">
         <v>595</v>
       </c>
       <c r="Q71" s="6">
@@ -9426,7 +9518,7 @@
       <c r="O72" s="4">
         <v>426</v>
       </c>
-      <c r="P72" s="47">
+      <c r="P72" s="44">
         <v>595</v>
       </c>
       <c r="Q72" s="6">
@@ -9488,7 +9580,7 @@
       <c r="O73" s="4">
         <v>360</v>
       </c>
-      <c r="P73" s="47">
+      <c r="P73" s="44">
         <v>495</v>
       </c>
       <c r="Q73" s="6">
@@ -9550,7 +9642,7 @@
       <c r="O74" s="4">
         <v>208</v>
       </c>
-      <c r="P74" s="47">
+      <c r="P74" s="44">
         <v>695</v>
       </c>
       <c r="Q74" s="6">
@@ -9612,7 +9704,7 @@
       <c r="O75" s="4">
         <v>518</v>
       </c>
-      <c r="P75" s="47">
+      <c r="P75" s="44">
         <v>445</v>
       </c>
       <c r="Q75" s="6">
@@ -9674,7 +9766,7 @@
       <c r="O76" s="4">
         <v>274</v>
       </c>
-      <c r="P76" s="47">
+      <c r="P76" s="44">
         <v>295</v>
       </c>
       <c r="Q76" s="6">
@@ -9736,7 +9828,7 @@
       <c r="O77" s="4">
         <v>216</v>
       </c>
-      <c r="P77" s="47">
+      <c r="P77" s="44">
         <v>395</v>
       </c>
       <c r="Q77" s="6">
@@ -9798,7 +9890,7 @@
       <c r="O78" s="4">
         <v>274</v>
       </c>
-      <c r="P78" s="47">
+      <c r="P78" s="44">
         <v>650</v>
       </c>
       <c r="Q78" s="6">
@@ -9860,7 +9952,7 @@
       <c r="O79" s="4">
         <v>606</v>
       </c>
-      <c r="P79" s="47">
+      <c r="P79" s="44">
         <v>1295</v>
       </c>
       <c r="Q79" s="6">
@@ -9922,7 +10014,7 @@
       <c r="O80" s="4">
         <v>350</v>
       </c>
-      <c r="P80" s="47">
+      <c r="P80" s="44">
         <v>950</v>
       </c>
       <c r="Q80" s="6">
@@ -9984,7 +10076,7 @@
       <c r="O81" s="4">
         <v>270</v>
       </c>
-      <c r="P81" s="47">
+      <c r="P81" s="44">
         <v>695</v>
       </c>
       <c r="Q81" s="6">
@@ -10046,7 +10138,7 @@
       <c r="O82" s="4">
         <v>292</v>
       </c>
-      <c r="P82" s="47">
+      <c r="P82" s="44">
         <v>795</v>
       </c>
       <c r="Q82" s="6">
@@ -10108,7 +10200,7 @@
       <c r="O83" s="4">
         <v>890</v>
       </c>
-      <c r="P83" s="47">
+      <c r="P83" s="44">
         <v>525</v>
       </c>
       <c r="Q83" s="6">
@@ -10170,7 +10262,7 @@
       <c r="O84" s="4">
         <v>144</v>
       </c>
-      <c r="P84" s="47">
+      <c r="P84" s="44">
         <v>225</v>
       </c>
       <c r="Q84" s="6">
@@ -10232,7 +10324,7 @@
       <c r="O85" s="4">
         <v>338</v>
       </c>
-      <c r="P85" s="47">
+      <c r="P85" s="44">
         <v>695</v>
       </c>
       <c r="Q85" s="6">
@@ -10294,7 +10386,7 @@
       <c r="O86" s="4">
         <v>432</v>
       </c>
-      <c r="P86" s="47">
+      <c r="P86" s="44">
         <v>550</v>
       </c>
       <c r="Q86" s="6">
@@ -10356,7 +10448,7 @@
       <c r="O87" s="4">
         <v>306</v>
       </c>
-      <c r="P87" s="47">
+      <c r="P87" s="44">
         <v>345</v>
       </c>
       <c r="Q87" s="6">
@@ -10418,7 +10510,7 @@
       <c r="O88" s="4">
         <v>172</v>
       </c>
-      <c r="P88" s="47">
+      <c r="P88" s="44">
         <v>350</v>
       </c>
       <c r="Q88" s="6">
@@ -10480,7 +10572,7 @@
       <c r="O89" s="4">
         <v>604</v>
       </c>
-      <c r="P89" s="47">
+      <c r="P89" s="44">
         <v>1195</v>
       </c>
       <c r="Q89" s="6">
@@ -10542,7 +10634,7 @@
       <c r="O90" s="4">
         <v>598</v>
       </c>
-      <c r="P90" s="47">
+      <c r="P90" s="44">
         <v>550</v>
       </c>
       <c r="Q90" s="6">
@@ -10604,7 +10696,7 @@
       <c r="O91" s="4">
         <v>878</v>
       </c>
-      <c r="P91" s="47">
+      <c r="P91" s="44">
         <v>695</v>
       </c>
       <c r="Q91" s="6">
@@ -10666,7 +10758,7 @@
       <c r="O92" s="4">
         <v>234</v>
       </c>
-      <c r="P92" s="47">
+      <c r="P92" s="44">
         <v>695</v>
       </c>
       <c r="Q92" s="6">
@@ -10728,7 +10820,7 @@
       <c r="O93" s="4">
         <v>476</v>
       </c>
-      <c r="P93" s="47">
+      <c r="P93" s="44">
         <v>595</v>
       </c>
       <c r="Q93" s="6">
@@ -10790,7 +10882,7 @@
       <c r="O94" s="4">
         <v>322</v>
       </c>
-      <c r="P94" s="47">
+      <c r="P94" s="44">
         <v>695</v>
       </c>
       <c r="Q94" s="6">
@@ -10852,7 +10944,7 @@
       <c r="O95" s="4">
         <v>288</v>
       </c>
-      <c r="P95" s="47">
+      <c r="P95" s="44">
         <v>695</v>
       </c>
       <c r="Q95" s="6">
@@ -10914,7 +11006,7 @@
       <c r="O96" s="4">
         <v>358</v>
       </c>
-      <c r="P96" s="47">
+      <c r="P96" s="44">
         <v>795</v>
       </c>
       <c r="Q96" s="6">
@@ -10976,7 +11068,7 @@
       <c r="O97" s="4">
         <v>380</v>
       </c>
-      <c r="P97" s="47">
+      <c r="P97" s="44">
         <v>475</v>
       </c>
       <c r="Q97" s="6">
@@ -11038,7 +11130,7 @@
       <c r="O98" s="4">
         <v>424</v>
       </c>
-      <c r="P98" s="47">
+      <c r="P98" s="44">
         <v>525</v>
       </c>
       <c r="Q98" s="6">
@@ -11100,7 +11192,7 @@
       <c r="O99" s="4">
         <v>348</v>
       </c>
-      <c r="P99" s="47">
+      <c r="P99" s="44">
         <v>325</v>
       </c>
       <c r="Q99" s="6">
@@ -11162,7 +11254,7 @@
       <c r="O100" s="4">
         <v>426</v>
       </c>
-      <c r="P100" s="47">
+      <c r="P100" s="44">
         <v>495</v>
       </c>
       <c r="Q100" s="6">
@@ -11224,7 +11316,7 @@
       <c r="O101" s="4">
         <v>598</v>
       </c>
-      <c r="P101" s="47">
+      <c r="P101" s="44">
         <v>595</v>
       </c>
       <c r="Q101" s="6">
@@ -11286,7 +11378,7 @@
       <c r="O102" s="4">
         <v>1954</v>
       </c>
-      <c r="P102" s="47">
+      <c r="P102" s="44">
         <v>4995</v>
       </c>
       <c r="Q102" s="6">
@@ -11348,7 +11440,7 @@
       <c r="O103" s="4">
         <v>354</v>
       </c>
-      <c r="P103" s="47">
+      <c r="P103" s="44">
         <v>425</v>
       </c>
       <c r="Q103" s="6">
@@ -11410,7 +11502,7 @@
       <c r="O104" s="4">
         <v>778</v>
       </c>
-      <c r="P104" s="47">
+      <c r="P104" s="44">
         <v>495</v>
       </c>
       <c r="Q104" s="6">
@@ -11472,7 +11564,7 @@
       <c r="O105" s="4">
         <v>334</v>
       </c>
-      <c r="P105" s="47">
+      <c r="P105" s="44">
         <v>795</v>
       </c>
       <c r="Q105" s="6">
@@ -11534,7 +11626,7 @@
       <c r="O106" s="4">
         <v>256</v>
       </c>
-      <c r="P106" s="47">
+      <c r="P106" s="44">
         <v>795</v>
       </c>
       <c r="Q106" s="6">
@@ -11596,7 +11688,7 @@
       <c r="O107" s="4">
         <v>330</v>
       </c>
-      <c r="P107" s="47">
+      <c r="P107" s="44">
         <v>1250</v>
       </c>
       <c r="Q107" s="6">
@@ -11658,7 +11750,7 @@
       <c r="O108" s="4">
         <v>216</v>
       </c>
-      <c r="P108" s="47">
+      <c r="P108" s="44">
         <v>245</v>
       </c>
       <c r="Q108" s="6">
@@ -11720,7 +11812,7 @@
       <c r="O109" s="4">
         <v>682</v>
       </c>
-      <c r="P109" s="47">
+      <c r="P109" s="44">
         <v>540</v>
       </c>
       <c r="Q109" s="6">
@@ -11782,7 +11874,7 @@
       <c r="O110" s="4">
         <v>470</v>
       </c>
-      <c r="P110" s="47">
+      <c r="P110" s="44">
         <v>550</v>
       </c>
       <c r="Q110" s="6">
@@ -11844,7 +11936,7 @@
       <c r="O111" s="4">
         <v>604</v>
       </c>
-      <c r="P111" s="47">
+      <c r="P111" s="44">
         <v>695</v>
       </c>
       <c r="Q111" s="6">
@@ -11906,7 +11998,7 @@
       <c r="O112" s="4">
         <v>350</v>
       </c>
-      <c r="P112" s="47">
+      <c r="P112" s="44">
         <v>795</v>
       </c>
       <c r="Q112" s="6">
@@ -11968,7 +12060,7 @@
       <c r="O113" s="4">
         <v>442</v>
       </c>
-      <c r="P113" s="47">
+      <c r="P113" s="44">
         <v>895</v>
       </c>
       <c r="Q113" s="6">
@@ -12030,7 +12122,7 @@
       <c r="O114" s="4">
         <v>350</v>
       </c>
-      <c r="P114" s="47">
+      <c r="P114" s="44">
         <v>895</v>
       </c>
       <c r="Q114" s="6">
@@ -12092,7 +12184,7 @@
       <c r="O115" s="4">
         <v>276</v>
       </c>
-      <c r="P115" s="47">
+      <c r="P115" s="44">
         <v>350</v>
       </c>
       <c r="Q115" s="6">
@@ -12154,7 +12246,7 @@
       <c r="O116" s="4">
         <v>282</v>
       </c>
-      <c r="P116" s="47">
+      <c r="P116" s="44">
         <v>350</v>
       </c>
       <c r="Q116" s="6">
@@ -12216,7 +12308,7 @@
       <c r="O117" s="4">
         <v>478</v>
       </c>
-      <c r="P117" s="47">
+      <c r="P117" s="44">
         <v>395</v>
       </c>
       <c r="Q117" s="6">
@@ -12278,7 +12370,7 @@
       <c r="O118" s="4">
         <v>512</v>
       </c>
-      <c r="P118" s="47">
+      <c r="P118" s="44">
         <v>495</v>
       </c>
       <c r="Q118" s="6">
@@ -12340,7 +12432,7 @@
       <c r="O119" s="4">
         <v>498</v>
       </c>
-      <c r="P119" s="47">
+      <c r="P119" s="44">
         <v>395</v>
       </c>
       <c r="Q119" s="6">
@@ -12402,7 +12494,7 @@
       <c r="O120" s="4">
         <v>288</v>
       </c>
-      <c r="P120" s="47">
+      <c r="P120" s="44">
         <v>350</v>
       </c>
       <c r="Q120" s="6">
@@ -12464,7 +12556,7 @@
       <c r="O121" s="4">
         <v>224</v>
       </c>
-      <c r="P121" s="47">
+      <c r="P121" s="44">
         <v>595</v>
       </c>
       <c r="Q121" s="6">
@@ -12526,7 +12618,7 @@
       <c r="O122" s="4">
         <v>670</v>
       </c>
-      <c r="P122" s="47">
+      <c r="P122" s="44">
         <v>525</v>
       </c>
       <c r="Q122" s="6">
@@ -12588,7 +12680,7 @@
       <c r="O123" s="4">
         <v>360</v>
       </c>
-      <c r="P123" s="47">
+      <c r="P123" s="44">
         <v>595</v>
       </c>
       <c r="Q123" s="6">
@@ -12650,7 +12742,7 @@
       <c r="O124" s="4">
         <v>412</v>
       </c>
-      <c r="P124" s="47">
+      <c r="P124" s="44">
         <v>525</v>
       </c>
       <c r="Q124" s="6">
@@ -12712,7 +12804,7 @@
       <c r="O125" s="4">
         <v>958</v>
       </c>
-      <c r="P125" s="47">
+      <c r="P125" s="44">
         <v>2250</v>
       </c>
       <c r="Q125" s="6">
@@ -12774,7 +12866,7 @@
       <c r="O126" s="4">
         <v>368</v>
       </c>
-      <c r="P126" s="47">
+      <c r="P126" s="44">
         <v>795</v>
       </c>
       <c r="Q126" s="6">
@@ -12836,7 +12928,7 @@
       <c r="O127" s="4">
         <v>362</v>
       </c>
-      <c r="P127" s="47">
+      <c r="P127" s="44">
         <v>350</v>
       </c>
       <c r="Q127" s="6">
@@ -12898,7 +12990,7 @@
       <c r="O128" s="4">
         <v>452</v>
       </c>
-      <c r="P128" s="47">
+      <c r="P128" s="44">
         <v>1195</v>
       </c>
       <c r="Q128" s="6">
@@ -12960,7 +13052,7 @@
       <c r="O129" s="4">
         <v>174</v>
       </c>
-      <c r="P129" s="47">
+      <c r="P129" s="44">
         <v>395</v>
       </c>
       <c r="Q129" s="6">
@@ -13022,7 +13114,7 @@
       <c r="O130" s="4">
         <v>32</v>
       </c>
-      <c r="P130" s="47">
+      <c r="P130" s="44">
         <v>175</v>
       </c>
       <c r="Q130" s="6">
@@ -13084,7 +13176,7 @@
       <c r="O131" s="4">
         <v>246</v>
       </c>
-      <c r="P131" s="47">
+      <c r="P131" s="44">
         <v>695</v>
       </c>
       <c r="Q131" s="6">
@@ -13146,7 +13238,7 @@
       <c r="O132" s="4">
         <v>178</v>
       </c>
-      <c r="P132" s="47">
+      <c r="P132" s="44">
         <v>650</v>
       </c>
       <c r="Q132" s="6">
@@ -13208,7 +13300,7 @@
       <c r="O133" s="4">
         <v>2652</v>
       </c>
-      <c r="P133" s="47">
+      <c r="P133" s="44">
         <v>3850</v>
       </c>
       <c r="Q133" s="6">
@@ -13270,7 +13362,7 @@
       <c r="O134" s="4">
         <v>340</v>
       </c>
-      <c r="P134" s="47">
+      <c r="P134" s="44">
         <v>995</v>
       </c>
       <c r="Q134" s="6">
@@ -13332,7 +13424,7 @@
       <c r="O135" s="4">
         <v>360</v>
       </c>
-      <c r="P135" s="47">
+      <c r="P135" s="44">
         <v>795</v>
       </c>
       <c r="Q135" s="6">
@@ -13394,7 +13486,7 @@
       <c r="O136" s="4">
         <v>852</v>
       </c>
-      <c r="P136" s="47">
+      <c r="P136" s="44">
         <v>795</v>
       </c>
       <c r="Q136" s="6">
@@ -13456,7 +13548,7 @@
       <c r="O137" s="4">
         <v>224</v>
       </c>
-      <c r="P137" s="47">
+      <c r="P137" s="44">
         <v>295</v>
       </c>
       <c r="Q137" s="6">
@@ -13518,7 +13610,7 @@
       <c r="O138" s="4">
         <v>474</v>
       </c>
-      <c r="P138" s="47">
+      <c r="P138" s="44">
         <v>470</v>
       </c>
       <c r="Q138" s="6">
@@ -13580,7 +13672,7 @@
       <c r="O139" s="4">
         <v>242</v>
       </c>
-      <c r="P139" s="47">
+      <c r="P139" s="44">
         <v>995</v>
       </c>
       <c r="Q139" s="6">
@@ -13642,7 +13734,7 @@
       <c r="O140" s="4">
         <v>182</v>
       </c>
-      <c r="P140" s="47">
+      <c r="P140" s="44">
         <v>230</v>
       </c>
       <c r="Q140" s="6">
@@ -13704,7 +13796,7 @@
       <c r="O141" s="4">
         <v>222</v>
       </c>
-      <c r="P141" s="47">
+      <c r="P141" s="44">
         <v>350</v>
       </c>
       <c r="Q141" s="6">
@@ -13766,7 +13858,7 @@
       <c r="O142" s="4">
         <v>694</v>
       </c>
-      <c r="P142" s="47">
+      <c r="P142" s="44">
         <v>895</v>
       </c>
       <c r="Q142" s="6">
@@ -13828,7 +13920,7 @@
       <c r="O143" s="4">
         <v>653</v>
       </c>
-      <c r="P143" s="47">
+      <c r="P143" s="44">
         <v>595</v>
       </c>
       <c r="Q143" s="6">
@@ -13890,7 +13982,7 @@
       <c r="O144" s="4">
         <v>390</v>
       </c>
-      <c r="P144" s="47">
+      <c r="P144" s="44">
         <v>395</v>
       </c>
       <c r="Q144" s="6">
@@ -13952,7 +14044,7 @@
       <c r="O145" s="4">
         <v>238</v>
       </c>
-      <c r="P145" s="47">
+      <c r="P145" s="44">
         <v>795</v>
       </c>
       <c r="Q145" s="6">
@@ -14014,7 +14106,7 @@
       <c r="O146" s="4">
         <v>506</v>
       </c>
-      <c r="P146" s="47">
+      <c r="P146" s="44">
         <v>525</v>
       </c>
       <c r="Q146" s="6">
@@ -14076,7 +14168,7 @@
       <c r="O147" s="4">
         <v>318</v>
       </c>
-      <c r="P147" s="47">
+      <c r="P147" s="44">
         <v>350</v>
       </c>
       <c r="Q147" s="6">
@@ -14138,7 +14230,7 @@
       <c r="O148" s="4">
         <v>454</v>
       </c>
-      <c r="P148" s="47">
+      <c r="P148" s="44">
         <v>495</v>
       </c>
       <c r="Q148" s="6">
@@ -14200,7 +14292,7 @@
       <c r="O149" s="4">
         <v>141</v>
       </c>
-      <c r="P149" s="47">
+      <c r="P149" s="44">
         <v>299</v>
       </c>
       <c r="Q149" s="6">
@@ -14262,7 +14354,7 @@
       <c r="O150" s="4">
         <v>816</v>
       </c>
-      <c r="P150" s="47">
+      <c r="P150" s="44">
         <v>795</v>
       </c>
       <c r="Q150" s="6">
@@ -14324,7 +14416,7 @@
       <c r="O151" s="4">
         <v>972</v>
       </c>
-      <c r="P151" s="47">
+      <c r="P151" s="44">
         <v>2100</v>
       </c>
       <c r="Q151" s="6">
@@ -14386,7 +14478,7 @@
       <c r="O152" s="4">
         <v>264</v>
       </c>
-      <c r="P152" s="47">
+      <c r="P152" s="44">
         <v>595</v>
       </c>
       <c r="Q152" s="6">
@@ -14448,7 +14540,7 @@
       <c r="O153" s="4">
         <v>410</v>
       </c>
-      <c r="P153" s="47">
+      <c r="P153" s="44">
         <v>695</v>
       </c>
       <c r="Q153" s="6">
@@ -14510,7 +14602,7 @@
       <c r="O154" s="4">
         <v>532</v>
       </c>
-      <c r="P154" s="47">
+      <c r="P154" s="44">
         <v>895</v>
       </c>
       <c r="Q154" s="6">
@@ -14572,7 +14664,7 @@
       <c r="O155" s="4">
         <v>516</v>
       </c>
-      <c r="P155" s="47">
+      <c r="P155" s="44">
         <v>995</v>
       </c>
       <c r="Q155" s="6">
@@ -14634,7 +14726,7 @@
       <c r="O156" s="4">
         <v>300</v>
       </c>
-      <c r="P156" s="47">
+      <c r="P156" s="44">
         <v>595</v>
       </c>
       <c r="Q156" s="6">
@@ -14696,7 +14788,7 @@
       <c r="O157" s="4">
         <v>2644</v>
       </c>
-      <c r="P157" s="47">
+      <c r="P157" s="44">
         <v>4995</v>
       </c>
       <c r="Q157" s="6">
@@ -14758,7 +14850,7 @@
       <c r="O158" s="4">
         <v>320</v>
       </c>
-      <c r="P158" s="47">
+      <c r="P158" s="44">
         <v>1250</v>
       </c>
       <c r="Q158" s="6">
@@ -14820,7 +14912,7 @@
       <c r="O159" s="4">
         <v>292</v>
       </c>
-      <c r="P159" s="47">
+      <c r="P159" s="44">
         <v>350</v>
       </c>
       <c r="Q159" s="6">
@@ -14882,7 +14974,7 @@
       <c r="O160" s="4">
         <v>404</v>
       </c>
-      <c r="P160" s="47">
+      <c r="P160" s="44">
         <v>895</v>
       </c>
       <c r="Q160" s="6">
@@ -14944,7 +15036,7 @@
       <c r="O161" s="4">
         <v>402</v>
       </c>
-      <c r="P161" s="47">
+      <c r="P161" s="44">
         <v>850</v>
       </c>
       <c r="Q161" s="6">
@@ -15006,7 +15098,7 @@
       <c r="O162" s="4">
         <v>1754</v>
       </c>
-      <c r="P162" s="47">
+      <c r="P162" s="44">
         <v>4450</v>
       </c>
       <c r="Q162" s="6">
@@ -15068,7 +15160,7 @@
       <c r="O163" s="4">
         <v>398</v>
       </c>
-      <c r="P163" s="47">
+      <c r="P163" s="44">
         <v>695</v>
       </c>
       <c r="Q163" s="6">
@@ -15130,7 +15222,7 @@
       <c r="O164" s="4">
         <v>216</v>
       </c>
-      <c r="P164" s="47">
+      <c r="P164" s="44">
         <v>300</v>
       </c>
       <c r="Q164" s="6">
@@ -15192,7 +15284,7 @@
       <c r="O165" s="4">
         <v>700</v>
       </c>
-      <c r="P165" s="47">
+      <c r="P165" s="44">
         <v>570</v>
       </c>
       <c r="Q165" s="6">
@@ -15254,7 +15346,7 @@
       <c r="O166" s="4">
         <v>228</v>
       </c>
-      <c r="P166" s="47">
+      <c r="P166" s="44">
         <v>695</v>
       </c>
       <c r="Q166" s="6">
@@ -15316,7 +15408,7 @@
       <c r="O167" s="4">
         <v>218</v>
       </c>
-      <c r="P167" s="47">
+      <c r="P167" s="44">
         <v>495</v>
       </c>
       <c r="Q167" s="6">
@@ -15378,7 +15470,7 @@
       <c r="O168" s="4">
         <v>197</v>
       </c>
-      <c r="P168" s="47">
+      <c r="P168" s="44">
         <v>495</v>
       </c>
       <c r="Q168" s="6">
@@ -15440,7 +15532,7 @@
       <c r="O169" s="4">
         <v>184</v>
       </c>
-      <c r="P169" s="47">
+      <c r="P169" s="44">
         <v>495</v>
       </c>
       <c r="Q169" s="6">
@@ -15502,7 +15594,7 @@
       <c r="O170" s="4">
         <v>456</v>
       </c>
-      <c r="P170" s="47">
+      <c r="P170" s="44">
         <v>495</v>
       </c>
       <c r="Q170" s="6">
@@ -15564,7 +15656,7 @@
       <c r="O171" s="4">
         <v>570</v>
       </c>
-      <c r="P171" s="47">
+      <c r="P171" s="44">
         <v>595</v>
       </c>
       <c r="Q171" s="6">
@@ -15626,7 +15718,7 @@
       <c r="O172" s="4">
         <v>238</v>
       </c>
-      <c r="P172" s="47">
+      <c r="P172" s="44">
         <v>395</v>
       </c>
       <c r="Q172" s="6">
@@ -15688,7 +15780,7 @@
       <c r="O173" s="4">
         <v>2814</v>
       </c>
-      <c r="P173" s="47">
+      <c r="P173" s="44">
         <v>4250</v>
       </c>
       <c r="Q173" s="6">
@@ -15750,7 +15842,7 @@
       <c r="O174" s="4">
         <v>448</v>
       </c>
-      <c r="P174" s="47">
+      <c r="P174" s="44">
         <v>1050</v>
       </c>
       <c r="Q174" s="6">
@@ -15812,7 +15904,7 @@
       <c r="O175" s="4">
         <v>702</v>
       </c>
-      <c r="P175" s="47">
+      <c r="P175" s="44">
         <v>565</v>
       </c>
       <c r="Q175" s="6">
@@ -15874,7 +15966,7 @@
       <c r="O176" s="4">
         <v>454</v>
       </c>
-      <c r="P176" s="47">
+      <c r="P176" s="44">
         <v>1195</v>
       </c>
       <c r="Q176" s="6">
@@ -15936,7 +16028,7 @@
       <c r="O177" s="4">
         <v>432</v>
       </c>
-      <c r="P177" s="47">
+      <c r="P177" s="44">
         <v>595</v>
       </c>
       <c r="Q177" s="6">
@@ -15998,7 +16090,7 @@
       <c r="O178" s="4">
         <v>276</v>
       </c>
-      <c r="P178" s="47">
+      <c r="P178" s="44">
         <v>495</v>
       </c>
       <c r="Q178" s="6">
@@ -16060,7 +16152,7 @@
       <c r="O179" s="4">
         <v>256</v>
       </c>
-      <c r="P179" s="47">
+      <c r="P179" s="44">
         <v>350</v>
       </c>
       <c r="Q179" s="6">
@@ -16122,7 +16214,7 @@
       <c r="O180" s="4">
         <v>1066</v>
       </c>
-      <c r="P180" s="47">
+      <c r="P180" s="44">
         <v>2495</v>
       </c>
       <c r="Q180" s="6">
@@ -16184,7 +16276,7 @@
       <c r="O181" s="4">
         <v>272</v>
       </c>
-      <c r="P181" s="47">
+      <c r="P181" s="44">
         <v>595</v>
       </c>
       <c r="Q181" s="6">
@@ -16246,7 +16338,7 @@
       <c r="O182" s="4">
         <v>552</v>
       </c>
-      <c r="P182" s="47">
+      <c r="P182" s="44">
         <v>995</v>
       </c>
       <c r="Q182" s="6">
@@ -16308,7 +16400,7 @@
       <c r="O183" s="4">
         <v>235</v>
       </c>
-      <c r="P183" s="47">
+      <c r="P183" s="44">
         <v>495</v>
       </c>
       <c r="Q183" s="6">
@@ -16370,7 +16462,7 @@
       <c r="O184" s="4">
         <v>414</v>
       </c>
-      <c r="P184" s="47">
+      <c r="P184" s="44">
         <v>1050</v>
       </c>
       <c r="Q184" s="6">
@@ -16432,7 +16524,7 @@
       <c r="O185" s="4">
         <v>414</v>
       </c>
-      <c r="P185" s="47">
+      <c r="P185" s="44">
         <v>895</v>
       </c>
       <c r="Q185" s="6">
@@ -16494,7 +16586,7 @@
       <c r="O186" s="4">
         <v>826</v>
       </c>
-      <c r="P186" s="47">
+      <c r="P186" s="44">
         <v>1995</v>
       </c>
       <c r="Q186" s="6">
@@ -16556,7 +16648,7 @@
       <c r="O187" s="4">
         <v>212</v>
       </c>
-      <c r="P187" s="47">
+      <c r="P187" s="44">
         <v>695</v>
       </c>
       <c r="Q187" s="6">
@@ -16618,7 +16710,7 @@
       <c r="O188" s="4">
         <v>396</v>
       </c>
-      <c r="P188" s="47">
+      <c r="P188" s="44">
         <v>1495</v>
       </c>
       <c r="Q188" s="6">
@@ -16680,7 +16772,7 @@
       <c r="O189" s="4">
         <v>324</v>
       </c>
-      <c r="P189" s="47">
+      <c r="P189" s="44">
         <v>995</v>
       </c>
       <c r="Q189" s="6">
@@ -16742,7 +16834,7 @@
       <c r="O190" s="4">
         <v>1084</v>
       </c>
-      <c r="P190" s="47">
+      <c r="P190" s="44">
         <v>2995</v>
       </c>
       <c r="Q190" s="6">
@@ -16804,7 +16896,7 @@
       <c r="O191" s="4">
         <v>250</v>
       </c>
-      <c r="P191" s="47">
+      <c r="P191" s="44">
         <v>795</v>
       </c>
       <c r="Q191" s="6">
@@ -16866,7 +16958,7 @@
       <c r="O192" s="4">
         <v>566</v>
       </c>
-      <c r="P192" s="47">
+      <c r="P192" s="44">
         <v>595</v>
       </c>
       <c r="Q192" s="6">
@@ -16928,7 +17020,7 @@
       <c r="O193" s="4">
         <v>2028</v>
       </c>
-      <c r="P193" s="47">
+      <c r="P193" s="44">
         <v>4495</v>
       </c>
       <c r="Q193" s="6">
@@ -16990,7 +17082,7 @@
       <c r="O194" s="4">
         <v>310</v>
       </c>
-      <c r="P194" s="47">
+      <c r="P194" s="44">
         <v>595</v>
       </c>
       <c r="Q194" s="6">
@@ -17052,7 +17144,7 @@
       <c r="O195" s="4">
         <v>768</v>
       </c>
-      <c r="P195" s="47">
+      <c r="P195" s="44">
         <v>1695</v>
       </c>
       <c r="Q195" s="6">
@@ -17114,7 +17206,7 @@
       <c r="O196" s="4">
         <v>378</v>
       </c>
-      <c r="P196" s="47">
+      <c r="P196" s="44">
         <v>450</v>
       </c>
       <c r="Q196" s="6">
@@ -17176,7 +17268,7 @@
       <c r="O197" s="4">
         <v>258</v>
       </c>
-      <c r="P197" s="47">
+      <c r="P197" s="44">
         <v>595</v>
       </c>
       <c r="Q197" s="6">
@@ -17238,7 +17330,7 @@
       <c r="O198" s="4">
         <v>1058</v>
       </c>
-      <c r="P198" s="47">
+      <c r="P198" s="44">
         <v>2495</v>
       </c>
       <c r="Q198" s="6">
@@ -17300,7 +17392,7 @@
       <c r="O199" s="4">
         <v>758</v>
       </c>
-      <c r="P199" s="47">
+      <c r="P199" s="44">
         <v>695</v>
       </c>
       <c r="Q199" s="6">
@@ -17362,7 +17454,7 @@
       <c r="O200" s="4">
         <v>286</v>
       </c>
-      <c r="P200" s="47">
+      <c r="P200" s="44">
         <v>695</v>
       </c>
       <c r="Q200" s="6">
@@ -17424,7 +17516,7 @@
       <c r="O201" s="4">
         <v>2686</v>
       </c>
-      <c r="P201" s="47">
+      <c r="P201" s="44">
         <v>4750</v>
       </c>
       <c r="Q201" s="6">
@@ -17486,7 +17578,7 @@
       <c r="O202" s="4">
         <v>200</v>
       </c>
-      <c r="P202" s="47">
+      <c r="P202" s="44">
         <v>695</v>
       </c>
       <c r="Q202" s="6">
@@ -17548,7 +17640,7 @@
       <c r="O203" s="4">
         <v>200</v>
       </c>
-      <c r="P203" s="47">
+      <c r="P203" s="44">
         <v>495</v>
       </c>
       <c r="Q203" s="6">
@@ -17610,7 +17702,7 @@
       <c r="O204" s="4">
         <v>1375</v>
       </c>
-      <c r="P204" s="47">
+      <c r="P204" s="44">
         <v>2995</v>
       </c>
       <c r="Q204" s="6">
@@ -17672,7 +17764,7 @@
       <c r="O205" s="4">
         <v>612</v>
       </c>
-      <c r="P205" s="47">
+      <c r="P205" s="44">
         <v>1395</v>
       </c>
       <c r="Q205" s="6">
@@ -17734,7 +17826,7 @@
       <c r="O206" s="4">
         <v>684</v>
       </c>
-      <c r="P206" s="47">
+      <c r="P206" s="44">
         <v>1550</v>
       </c>
       <c r="Q206" s="6">
@@ -17796,7 +17888,7 @@
       <c r="O207" s="4">
         <v>542</v>
       </c>
-      <c r="P207" s="47">
+      <c r="P207" s="44">
         <v>695</v>
       </c>
       <c r="Q207" s="6">
@@ -17858,7 +17950,7 @@
       <c r="O208" s="4">
         <v>516</v>
       </c>
-      <c r="P208" s="47">
+      <c r="P208" s="44">
         <v>750</v>
       </c>
       <c r="Q208" s="6">
@@ -17920,7 +18012,7 @@
       <c r="O209" s="4">
         <v>840</v>
       </c>
-      <c r="P209" s="47">
+      <c r="P209" s="44">
         <v>1795</v>
       </c>
       <c r="Q209" s="6">
@@ -17982,7 +18074,7 @@
       <c r="O210" s="4">
         <v>740</v>
       </c>
-      <c r="P210" s="47">
+      <c r="P210" s="44">
         <v>895</v>
       </c>
       <c r="Q210" s="6">
@@ -18044,7 +18136,7 @@
       <c r="O211" s="4">
         <v>460</v>
       </c>
-      <c r="P211" s="47">
+      <c r="P211" s="44">
         <v>450</v>
       </c>
       <c r="Q211" s="6">
@@ -18106,7 +18198,7 @@
       <c r="O212" s="4">
         <v>350</v>
       </c>
-      <c r="P212" s="47">
+      <c r="P212" s="44">
         <v>795</v>
       </c>
       <c r="Q212" s="6">
@@ -18168,7 +18260,7 @@
       <c r="O213" s="4">
         <v>428</v>
       </c>
-      <c r="P213" s="47">
+      <c r="P213" s="44">
         <v>995</v>
       </c>
       <c r="Q213" s="6">
@@ -18230,7 +18322,7 @@
       <c r="O214" s="4">
         <v>320</v>
       </c>
-      <c r="P214" s="47">
+      <c r="P214" s="44">
         <v>695</v>
       </c>
       <c r="Q214" s="6">
@@ -18292,7 +18384,7 @@
       <c r="O215" s="4">
         <v>16</v>
       </c>
-      <c r="P215" s="47">
+      <c r="P215" s="44">
         <v>295</v>
       </c>
       <c r="Q215" s="6">
@@ -18354,7 +18446,7 @@
       <c r="O216" s="4">
         <v>262</v>
       </c>
-      <c r="P216" s="47">
+      <c r="P216" s="44">
         <v>295</v>
       </c>
       <c r="Q216" s="6">
@@ -18416,7 +18508,7 @@
       <c r="O217" s="4">
         <v>2392</v>
       </c>
-      <c r="P217" s="47">
+      <c r="P217" s="44">
         <v>4995</v>
       </c>
       <c r="Q217" s="6">
@@ -18478,7 +18570,7 @@
       <c r="O218" s="4">
         <v>562</v>
       </c>
-      <c r="P218" s="47">
+      <c r="P218" s="44">
         <v>650</v>
       </c>
       <c r="Q218" s="6">
@@ -18540,7 +18632,7 @@
       <c r="O219" s="4">
         <v>226</v>
       </c>
-      <c r="P219" s="47">
+      <c r="P219" s="44">
         <v>495</v>
       </c>
       <c r="Q219" s="6">
@@ -18602,7 +18694,7 @@
       <c r="O220" s="6">
         <v>314</v>
       </c>
-      <c r="P220" s="48">
+      <c r="P220" s="45">
         <v>295</v>
       </c>
       <c r="Q220" s="6">
@@ -18664,7 +18756,7 @@
       <c r="O221" s="6">
         <v>1016</v>
       </c>
-      <c r="P221" s="48">
+      <c r="P221" s="45">
         <v>2495</v>
       </c>
       <c r="Q221" s="6">
@@ -18726,7 +18818,7 @@
       <c r="O222" s="6">
         <v>196</v>
       </c>
-      <c r="P222" s="48">
+      <c r="P222" s="45">
         <v>495</v>
       </c>
       <c r="Q222" s="6">
@@ -18788,7 +18880,7 @@
       <c r="O223" s="6">
         <v>284</v>
       </c>
-      <c r="P223" s="48">
+      <c r="P223" s="45">
         <v>695</v>
       </c>
       <c r="Q223" s="6">
@@ -18850,7 +18942,7 @@
       <c r="O224" s="6">
         <v>202</v>
       </c>
-      <c r="P224" s="48">
+      <c r="P224" s="45">
         <v>695</v>
       </c>
       <c r="Q224" s="6">
@@ -18912,7 +19004,7 @@
       <c r="O225" s="6">
         <v>242</v>
       </c>
-      <c r="P225" s="48">
+      <c r="P225" s="45">
         <v>495</v>
       </c>
       <c r="Q225" s="6">
@@ -18974,7 +19066,7 @@
       <c r="O226" s="6">
         <v>248</v>
       </c>
-      <c r="P226" s="48">
+      <c r="P226" s="45">
         <v>695</v>
       </c>
       <c r="Q226" s="6">
@@ -19036,7 +19128,7 @@
       <c r="O227" s="6">
         <v>390</v>
       </c>
-      <c r="P227" s="48">
+      <c r="P227" s="45">
         <v>795</v>
       </c>
       <c r="Q227" s="6">
@@ -19098,7 +19190,7 @@
       <c r="O228" s="6">
         <v>192</v>
       </c>
-      <c r="P228" s="48">
+      <c r="P228" s="45">
         <v>495</v>
       </c>
       <c r="Q228" s="6">
@@ -19160,7 +19252,7 @@
       <c r="O229" s="6">
         <v>148</v>
       </c>
-      <c r="P229" s="48">
+      <c r="P229" s="45">
         <v>450</v>
       </c>
       <c r="Q229" s="6">
@@ -19222,7 +19314,7 @@
       <c r="O230" s="6">
         <v>354</v>
       </c>
-      <c r="P230" s="48">
+      <c r="P230" s="45">
         <v>995</v>
       </c>
       <c r="Q230" s="6">
@@ -19284,7 +19376,7 @@
       <c r="O231" s="6">
         <v>926</v>
       </c>
-      <c r="P231" s="48">
+      <c r="P231" s="45">
         <v>1895</v>
       </c>
       <c r="Q231" s="6">
@@ -19346,7 +19438,7 @@
       <c r="O232" s="6">
         <v>510</v>
       </c>
-      <c r="P232" s="48">
+      <c r="P232" s="45">
         <v>995</v>
       </c>
       <c r="Q232" s="6">
@@ -19408,7 +19500,7 @@
       <c r="O233" s="6">
         <v>980</v>
       </c>
-      <c r="P233" s="48">
+      <c r="P233" s="45">
         <v>1895</v>
       </c>
       <c r="Q233" s="6">
@@ -19470,7 +19562,7 @@
       <c r="O234" s="6">
         <v>298</v>
       </c>
-      <c r="P234" s="48">
+      <c r="P234" s="45">
         <v>795</v>
       </c>
       <c r="Q234" s="6">
@@ -19532,7 +19624,7 @@
       <c r="O235" s="24">
         <v>766</v>
       </c>
-      <c r="P235" s="49">
+      <c r="P235" s="46">
         <v>625</v>
       </c>
       <c r="Q235" s="24">
@@ -19592,7 +19684,7 @@
       <c r="O236" s="24">
         <v>152</v>
       </c>
-      <c r="P236" s="49">
+      <c r="P236" s="46">
         <v>250</v>
       </c>
       <c r="Q236" s="24">
@@ -19652,7 +19744,7 @@
       <c r="O237" s="24">
         <v>188</v>
       </c>
-      <c r="P237" s="49">
+      <c r="P237" s="46">
         <v>295</v>
       </c>
       <c r="Q237" s="24">
@@ -19712,7 +19804,7 @@
       <c r="O238" s="24">
         <v>118</v>
       </c>
-      <c r="P238" s="49">
+      <c r="P238" s="46">
         <v>250</v>
       </c>
       <c r="Q238" s="24">
@@ -19772,7 +19864,7 @@
       <c r="O239" s="24">
         <v>226</v>
       </c>
-      <c r="P239" s="49">
+      <c r="P239" s="46">
         <v>595</v>
       </c>
       <c r="Q239" s="24" t="s">
@@ -19832,7 +19924,7 @@
       <c r="O240" s="24">
         <v>884</v>
       </c>
-      <c r="P240" s="49">
+      <c r="P240" s="46">
         <v>2495</v>
       </c>
       <c r="Q240" s="24">
@@ -19894,7 +19986,7 @@
       <c r="O241" s="24">
         <v>510</v>
       </c>
-      <c r="P241" s="49">
+      <c r="P241" s="46">
         <v>1295</v>
       </c>
       <c r="Q241" s="24">
@@ -19956,7 +20048,7 @@
       <c r="O242" s="6">
         <v>238</v>
       </c>
-      <c r="P242" s="48">
+      <c r="P242" s="45">
         <v>494</v>
       </c>
       <c r="Q242" s="6">
@@ -20016,7 +20108,7 @@
       <c r="O243" s="6">
         <v>794</v>
       </c>
-      <c r="P243" s="48">
+      <c r="P243" s="45">
         <v>750</v>
       </c>
       <c r="Q243" s="6" t="s">
@@ -20057,7 +20149,7 @@
       <c r="H244" s="7" t="s">
         <v>941</v>
       </c>
-      <c r="I244" s="45" t="s">
+      <c r="I244" s="42" t="s">
         <v>952</v>
       </c>
       <c r="J244" s="6">
@@ -20078,7 +20170,7 @@
       <c r="O244" s="6">
         <v>404</v>
       </c>
-      <c r="P244" s="48">
+      <c r="P244" s="45">
         <v>1095</v>
       </c>
       <c r="Q244" s="6">
@@ -20140,7 +20232,7 @@
       <c r="O245" s="6">
         <v>130</v>
       </c>
-      <c r="P245" s="48">
+      <c r="P245" s="45">
         <v>350</v>
       </c>
       <c r="Q245" s="6">
@@ -20178,10 +20270,10 @@
       <c r="G246" s="14" t="s">
         <v>930</v>
       </c>
-      <c r="H246" s="43" t="s">
+      <c r="H246" s="40" t="s">
         <v>948</v>
       </c>
-      <c r="I246" s="44" t="s">
+      <c r="I246" s="41" t="s">
         <v>949</v>
       </c>
       <c r="J246" s="6">
@@ -20202,7 +20294,7 @@
       <c r="O246" s="6">
         <v>702</v>
       </c>
-      <c r="P246" s="48">
+      <c r="P246" s="45">
         <v>1595</v>
       </c>
       <c r="Q246" s="6">
@@ -20219,64 +20311,64 @@
       </c>
     </row>
     <row r="247" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A247" s="6">
+      <c r="A247" s="51">
         <v>246</v>
       </c>
-      <c r="B247" s="6" t="s">
+      <c r="B247" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="C247" s="6" t="s">
+      <c r="C247" s="51" t="s">
         <v>148</v>
       </c>
-      <c r="D247" s="10">
+      <c r="D247" s="52">
         <v>9788199888142</v>
       </c>
-      <c r="E247" s="13" t="s">
+      <c r="E247" s="53" t="s">
         <v>934</v>
       </c>
-      <c r="F247" s="14" t="s">
+      <c r="F247" s="54" t="s">
         <v>933</v>
       </c>
-      <c r="G247" s="14" t="s">
+      <c r="G247" s="54" t="s">
         <v>932</v>
       </c>
-      <c r="H247" s="41" t="s">
+      <c r="H247" s="38" t="s">
         <v>946</v>
       </c>
-      <c r="I247" s="42" t="s">
+      <c r="I247" s="39" t="s">
         <v>947</v>
       </c>
-      <c r="J247" s="6">
+      <c r="J247" s="51">
         <v>1</v>
       </c>
-      <c r="K247" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="L247" s="6" t="s">
+      <c r="K247" s="51" t="s">
+        <v>219</v>
+      </c>
+      <c r="L247" s="51" t="s">
         <v>222</v>
       </c>
-      <c r="M247" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="N247" s="15">
+      <c r="M247" s="51" t="s">
+        <v>226</v>
+      </c>
+      <c r="N247" s="55">
         <v>46082</v>
       </c>
-      <c r="O247" s="6">
+      <c r="O247" s="51">
         <v>734</v>
       </c>
-      <c r="P247" s="48">
+      <c r="P247" s="56">
         <v>1845</v>
       </c>
-      <c r="Q247" s="6">
+      <c r="Q247" s="51">
         <v>24.8</v>
       </c>
-      <c r="R247" s="6">
+      <c r="R247" s="51">
         <v>16.3</v>
       </c>
-      <c r="S247" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="T247" s="6">
+      <c r="S247" s="51">
+        <v>2.5</v>
+      </c>
+      <c r="T247" s="51">
         <v>1050</v>
       </c>
     </row>
@@ -20302,10 +20394,10 @@
       <c r="G248" s="6" t="s">
         <v>938</v>
       </c>
-      <c r="H248" s="40" t="s">
+      <c r="H248" s="57" t="s">
         <v>944</v>
       </c>
-      <c r="I248" s="39" t="s">
+      <c r="I248" s="58" t="s">
         <v>945</v>
       </c>
       <c r="J248" s="6">
@@ -20326,7 +20418,7 @@
       <c r="O248" s="6">
         <v>244</v>
       </c>
-      <c r="P248" s="48">
+      <c r="P248" s="45">
         <v>695</v>
       </c>
       <c r="Q248" s="6">
@@ -20342,11 +20434,314 @@
         <v>260</v>
       </c>
     </row>
-    <row r="249" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="I249" s="38"/>
+    <row r="249" spans="1:20" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A249" s="9">
+        <v>248</v>
+      </c>
+      <c r="B249" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C249" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D249" s="48">
+        <v>9788199624559</v>
+      </c>
+      <c r="E249" s="9"/>
+      <c r="F249" s="9" t="s">
+        <v>955</v>
+      </c>
+      <c r="G249" s="9" t="s">
+        <v>954</v>
+      </c>
+      <c r="H249" s="59" t="s">
+        <v>964</v>
+      </c>
+      <c r="I249" s="60" t="s">
+        <v>965</v>
+      </c>
+      <c r="J249" s="9">
+        <v>1</v>
+      </c>
+      <c r="K249" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="L249" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="M249" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="N249" s="49">
+        <v>46143</v>
+      </c>
+      <c r="O249" s="9">
+        <v>231</v>
+      </c>
+      <c r="P249" s="50">
+        <v>595</v>
+      </c>
+      <c r="Q249" s="6">
+        <v>24</v>
+      </c>
+      <c r="R249" s="6">
+        <v>16</v>
+      </c>
+      <c r="S249" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="T249" s="9">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="250" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A250" s="9">
+        <v>249</v>
+      </c>
+      <c r="B250" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C250" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D250" s="48">
+        <v>9788199888173</v>
+      </c>
+      <c r="E250" s="9"/>
+      <c r="F250" s="9" t="s">
+        <v>731</v>
+      </c>
+      <c r="G250" s="9" t="s">
+        <v>956</v>
+      </c>
+      <c r="H250" s="59" t="s">
+        <v>621</v>
+      </c>
+      <c r="I250" s="60" t="s">
+        <v>963</v>
+      </c>
+      <c r="J250" s="9">
+        <v>1</v>
+      </c>
+      <c r="K250" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="L250" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="M250" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="N250" s="49">
+        <v>46143</v>
+      </c>
+      <c r="O250" s="9">
+        <v>2738</v>
+      </c>
+      <c r="P250" s="50">
+        <v>4800</v>
+      </c>
+      <c r="Q250" s="6">
+        <v>21.5</v>
+      </c>
+      <c r="R250" s="6">
+        <v>14</v>
+      </c>
+      <c r="S250" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="T250" s="9">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="251" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A251" s="9">
+        <v>251</v>
+      </c>
+      <c r="B251" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C251" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D251" s="48">
+        <v>9788199888159</v>
+      </c>
+      <c r="E251" s="9"/>
+      <c r="F251" s="9" t="s">
+        <v>747</v>
+      </c>
+      <c r="G251" s="9" t="s">
+        <v>953</v>
+      </c>
+      <c r="H251" s="59" t="s">
+        <v>959</v>
+      </c>
+      <c r="I251" s="61" t="s">
+        <v>960</v>
+      </c>
+      <c r="J251" s="9">
+        <v>2</v>
+      </c>
+      <c r="K251" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="L251" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="M251" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="N251" s="49">
+        <v>46204</v>
+      </c>
+      <c r="O251" s="9">
+        <v>572</v>
+      </c>
+      <c r="P251" s="50">
+        <v>795</v>
+      </c>
+      <c r="Q251" s="6">
+        <v>24</v>
+      </c>
+      <c r="R251" s="6">
+        <v>18.5</v>
+      </c>
+      <c r="S251" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="T251" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="252" spans="1:20" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A252" s="9">
+        <v>252</v>
+      </c>
+      <c r="B252" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C252" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D252" s="48">
+        <v>9788199888111</v>
+      </c>
+      <c r="E252" s="9"/>
+      <c r="F252" s="9" t="s">
+        <v>958</v>
+      </c>
+      <c r="G252" s="9" t="s">
+        <v>957</v>
+      </c>
+      <c r="H252" s="59" t="s">
+        <v>961</v>
+      </c>
+      <c r="I252" s="62" t="s">
+        <v>962</v>
+      </c>
+      <c r="J252" s="9">
+        <v>1</v>
+      </c>
+      <c r="K252" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="L252" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="M252" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="N252" s="49">
+        <v>46204</v>
+      </c>
+      <c r="O252" s="9">
+        <v>282</v>
+      </c>
+      <c r="P252" s="50">
+        <v>795</v>
+      </c>
+      <c r="Q252" s="6">
+        <v>24</v>
+      </c>
+      <c r="R252" s="6">
+        <v>16</v>
+      </c>
+      <c r="S252" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="T252" s="9">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="253" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A253" s="9"/>
+      <c r="B253" s="9"/>
+      <c r="C253" s="9"/>
+      <c r="D253" s="48"/>
+      <c r="E253" s="9"/>
+      <c r="F253" s="9"/>
+      <c r="G253" s="9"/>
+      <c r="H253" s="9"/>
+      <c r="I253" s="61"/>
+      <c r="J253" s="9"/>
+      <c r="K253" s="9"/>
+      <c r="L253" s="9"/>
+      <c r="M253" s="9"/>
+      <c r="N253" s="9"/>
+      <c r="O253" s="9"/>
+      <c r="P253" s="50"/>
+      <c r="Q253" s="9"/>
+      <c r="R253" s="9"/>
+      <c r="S253" s="9"/>
+      <c r="T253" s="9"/>
+    </row>
+    <row r="254" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A254" s="9"/>
+      <c r="B254" s="9"/>
+      <c r="C254" s="9"/>
+      <c r="D254" s="48"/>
+      <c r="E254" s="9"/>
+      <c r="F254" s="9"/>
+      <c r="G254" s="9"/>
+      <c r="H254" s="9"/>
+      <c r="I254" s="9"/>
+      <c r="J254" s="9"/>
+      <c r="K254" s="9"/>
+      <c r="L254" s="9"/>
+      <c r="M254" s="9"/>
+      <c r="N254" s="9"/>
+      <c r="O254" s="9"/>
+      <c r="P254" s="50"/>
+      <c r="Q254" s="9"/>
+      <c r="R254" s="9"/>
+      <c r="S254" s="9"/>
+      <c r="T254" s="9"/>
+    </row>
+    <row r="255" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A255" s="9"/>
+      <c r="B255" s="9"/>
+      <c r="C255" s="9"/>
+      <c r="D255" s="48"/>
+      <c r="E255" s="9"/>
+      <c r="F255" s="9"/>
+      <c r="G255" s="9"/>
+      <c r="H255" s="9"/>
+      <c r="I255" s="9"/>
+      <c r="J255" s="9"/>
+      <c r="K255" s="9"/>
+      <c r="L255" s="9"/>
+      <c r="M255" s="9"/>
+      <c r="N255" s="9"/>
+      <c r="O255" s="9"/>
+      <c r="P255" s="50"/>
+      <c r="Q255" s="9"/>
+      <c r="R255" s="9"/>
+      <c r="S255" s="9"/>
+      <c r="T255" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF248" xr:uid="{AAB18B99-872A-4F67-B7AF-943353254B42}">
+  <autoFilter ref="A1:AF252" xr:uid="{AAB18B99-872A-4F67-B7AF-943353254B42}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AF227">
       <sortCondition ref="A1"/>
     </sortState>

</xml_diff>